<commit_message>
Switch all tests to one-tailed; asterisks on p-values; NU/U results labels
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017FiZmvLfGJBDjNeFsfBt4t
</commit_message>
<xml_diff>
--- a/LastName_FirstName_U2P_Tables.xlsx
+++ b/LastName_FirstName_U2P_Tables.xlsx
@@ -2705,7 +2705,7 @@
       </c>
       <c r="I5" s="97" t="inlineStr">
         <is>
-          <t>.494</t>
+          <t>.247</t>
         </is>
       </c>
       <c r="J5" s="97" t="inlineStr"/>
@@ -2716,7 +2716,7 @@
       </c>
       <c r="L5" s="97" t="inlineStr">
         <is>
-          <t>.145</t>
+          <t>.073</t>
         </is>
       </c>
       <c r="M5" s="98" t="inlineStr"/>
@@ -2747,27 +2747,27 @@
       </c>
       <c r="H6" s="97" t="inlineStr">
         <is>
-          <t>-3.43***</t>
+          <t>-3.43</t>
         </is>
       </c>
       <c r="I6" s="97" t="inlineStr">
         <is>
-          <t>&lt;.001</t>
+          <t>&lt;.001***</t>
         </is>
       </c>
       <c r="J6" s="97" t="inlineStr">
         <is>
-          <t>U &gt; NU</t>
+          <t>NU &lt; U</t>
         </is>
       </c>
       <c r="K6" s="97" t="inlineStr">
         <is>
-          <t>1.50**</t>
+          <t>1.50</t>
         </is>
       </c>
       <c r="L6" s="97" t="inlineStr">
         <is>
-          <t>.001</t>
+          <t>&lt;.001***</t>
         </is>
       </c>
       <c r="M6" s="98" t="inlineStr">
@@ -2807,7 +2807,7 @@
       </c>
       <c r="I7" s="97" t="inlineStr">
         <is>
-          <t>.161</t>
+          <t>.081</t>
         </is>
       </c>
       <c r="J7" s="97" t="inlineStr"/>
@@ -2818,7 +2818,7 @@
       </c>
       <c r="L7" s="97" t="inlineStr">
         <is>
-          <t>.310</t>
+          <t>.155</t>
         </is>
       </c>
       <c r="M7" s="98" t="inlineStr"/>
@@ -2849,17 +2849,17 @@
       </c>
       <c r="H8" s="97" t="inlineStr">
         <is>
-          <t>-1.70†</t>
+          <t>-1.70</t>
         </is>
       </c>
       <c r="I8" s="97" t="inlineStr">
         <is>
-          <t>.090</t>
+          <t>.045*</t>
         </is>
       </c>
       <c r="J8" s="97" t="inlineStr">
         <is>
-          <t>U &gt; NU</t>
+          <t>NU &lt; U</t>
         </is>
       </c>
       <c r="K8" s="97" t="inlineStr">
@@ -2869,7 +2869,7 @@
       </c>
       <c r="L8" s="97" t="inlineStr">
         <is>
-          <t>.576</t>
+          <t>.288</t>
         </is>
       </c>
       <c r="M8" s="98" t="inlineStr"/>
@@ -2900,17 +2900,17 @@
       </c>
       <c r="H9" s="97" t="inlineStr">
         <is>
-          <t>-2.61**</t>
+          <t>-2.61</t>
         </is>
       </c>
       <c r="I9" s="97" t="inlineStr">
         <is>
-          <t>.009</t>
+          <t>.005**</t>
         </is>
       </c>
       <c r="J9" s="97" t="inlineStr">
         <is>
-          <t>U &gt; NU</t>
+          <t>NU &lt; U</t>
         </is>
       </c>
       <c r="K9" s="97" t="inlineStr">
@@ -2920,7 +2920,7 @@
       </c>
       <c r="L9" s="97" t="inlineStr">
         <is>
-          <t>.164</t>
+          <t>.082</t>
         </is>
       </c>
       <c r="M9" s="98" t="inlineStr"/>
@@ -2985,12 +2985,12 @@
       </c>
       <c r="H12" s="97" t="inlineStr">
         <is>
-          <t>4.25***</t>
+          <t>4.25</t>
         </is>
       </c>
       <c r="I12" s="97" t="inlineStr">
         <is>
-          <t>&lt;.001</t>
+          <t>&lt;.001***</t>
         </is>
       </c>
       <c r="J12" s="97" t="inlineStr">
@@ -3000,12 +3000,12 @@
       </c>
       <c r="K12" s="97" t="inlineStr">
         <is>
-          <t>1.85***</t>
+          <t>1.85</t>
         </is>
       </c>
       <c r="L12" s="97" t="inlineStr">
         <is>
-          <t>&lt;.001</t>
+          <t>&lt;.001***</t>
         </is>
       </c>
       <c r="M12" s="98" t="inlineStr">
@@ -3040,12 +3040,12 @@
       </c>
       <c r="H13" s="97" t="inlineStr">
         <is>
-          <t>1.69†</t>
+          <t>1.69</t>
         </is>
       </c>
       <c r="I13" s="97" t="inlineStr">
         <is>
-          <t>.092</t>
+          <t>.046*</t>
         </is>
       </c>
       <c r="J13" s="97" t="inlineStr">
@@ -3060,7 +3060,7 @@
       </c>
       <c r="L13" s="97" t="inlineStr">
         <is>
-          <t>.549</t>
+          <t>.275</t>
         </is>
       </c>
       <c r="M13" s="98" t="inlineStr"/>
@@ -3096,7 +3096,7 @@
       </c>
       <c r="I14" s="97" t="inlineStr">
         <is>
-          <t>.445</t>
+          <t>.222</t>
         </is>
       </c>
       <c r="J14" s="97" t="inlineStr"/>
@@ -3107,7 +3107,7 @@
       </c>
       <c r="L14" s="97" t="inlineStr">
         <is>
-          <t>.326</t>
+          <t>.163</t>
         </is>
       </c>
       <c r="M14" s="98" t="inlineStr"/>
@@ -3143,7 +3143,7 @@
       </c>
       <c r="I15" s="97" t="inlineStr">
         <is>
-          <t>.563</t>
+          <t>.281</t>
         </is>
       </c>
       <c r="J15" s="97" t="inlineStr"/>
@@ -3154,7 +3154,7 @@
       </c>
       <c r="L15" s="97" t="inlineStr">
         <is>
-          <t>.383</t>
+          <t>.191</t>
         </is>
       </c>
       <c r="M15" s="98" t="inlineStr"/>
@@ -3224,18 +3224,18 @@
       </c>
       <c r="I18" s="97" t="inlineStr">
         <is>
-          <t>.357</t>
+          <t>.179</t>
         </is>
       </c>
       <c r="J18" s="97" t="inlineStr"/>
       <c r="K18" s="97" t="inlineStr">
         <is>
-          <t>1.42**</t>
+          <t>1.42</t>
         </is>
       </c>
       <c r="L18" s="97" t="inlineStr">
         <is>
-          <t>.005</t>
+          <t>.003**</t>
         </is>
       </c>
       <c r="M18" s="98" t="inlineStr">
@@ -3270,27 +3270,27 @@
       </c>
       <c r="H19" s="97" t="inlineStr">
         <is>
-          <t>-1.79†</t>
+          <t>-1.79</t>
         </is>
       </c>
       <c r="I19" s="97" t="inlineStr">
         <is>
-          <t>.074</t>
+          <t>.037*</t>
         </is>
       </c>
       <c r="J19" s="97" t="inlineStr">
         <is>
-          <t>U &gt; NU</t>
+          <t>NU &lt; U</t>
         </is>
       </c>
       <c r="K19" s="97" t="inlineStr">
         <is>
-          <t>1.30*</t>
+          <t>1.30</t>
         </is>
       </c>
       <c r="L19" s="97" t="inlineStr">
         <is>
-          <t>.036</t>
+          <t>.018*</t>
         </is>
       </c>
       <c r="M19" s="98" t="inlineStr">
@@ -3325,27 +3325,27 @@
       </c>
       <c r="H20" s="97" t="inlineStr">
         <is>
-          <t>-2.73**</t>
+          <t>-2.73</t>
         </is>
       </c>
       <c r="I20" s="97" t="inlineStr">
         <is>
-          <t>.007</t>
+          <t>.003**</t>
         </is>
       </c>
       <c r="J20" s="97" t="inlineStr">
         <is>
-          <t>U &gt; NU</t>
+          <t>NU &lt; U</t>
         </is>
       </c>
       <c r="K20" s="97" t="inlineStr">
         <is>
-          <t>1.23†</t>
+          <t>1.23</t>
         </is>
       </c>
       <c r="L20" s="97" t="inlineStr">
         <is>
-          <t>.099</t>
+          <t>.050*</t>
         </is>
       </c>
       <c r="M20" s="98" t="inlineStr">
@@ -3385,7 +3385,7 @@
       </c>
       <c r="I21" s="97" t="inlineStr">
         <is>
-          <t>.315</t>
+          <t>.158</t>
         </is>
       </c>
       <c r="J21" s="97" t="inlineStr"/>
@@ -3396,7 +3396,7 @@
       </c>
       <c r="L21" s="97" t="inlineStr">
         <is>
-          <t>.309</t>
+          <t>.154</t>
         </is>
       </c>
       <c r="M21" s="98" t="inlineStr"/>
@@ -3427,27 +3427,27 @@
       </c>
       <c r="H22" s="97" t="inlineStr">
         <is>
-          <t>-3.42***</t>
+          <t>-3.42</t>
         </is>
       </c>
       <c r="I22" s="97" t="inlineStr">
         <is>
-          <t>&lt;.001</t>
+          <t>&lt;.001***</t>
         </is>
       </c>
       <c r="J22" s="97" t="inlineStr">
         <is>
-          <t>U &gt; NU</t>
+          <t>NU &lt; U</t>
         </is>
       </c>
       <c r="K22" s="97" t="inlineStr">
         <is>
-          <t>1.63***</t>
+          <t>1.63</t>
         </is>
       </c>
       <c r="L22" s="97" t="inlineStr">
         <is>
-          <t>&lt;.001</t>
+          <t>&lt;.001***</t>
         </is>
       </c>
       <c r="M22" s="98" t="inlineStr">
@@ -3482,27 +3482,27 @@
       </c>
       <c r="H23" s="97" t="inlineStr">
         <is>
-          <t>-2.99**</t>
+          <t>-2.99</t>
         </is>
       </c>
       <c r="I23" s="97" t="inlineStr">
         <is>
-          <t>.003</t>
+          <t>.001**</t>
         </is>
       </c>
       <c r="J23" s="97" t="inlineStr">
         <is>
-          <t>U &gt; NU</t>
+          <t>NU &lt; U</t>
         </is>
       </c>
       <c r="K23" s="97" t="inlineStr">
         <is>
-          <t>1.31*</t>
+          <t>1.31</t>
         </is>
       </c>
       <c r="L23" s="97" t="inlineStr">
         <is>
-          <t>.033</t>
+          <t>.017*</t>
         </is>
       </c>
       <c r="M23" s="98" t="inlineStr">
@@ -3537,12 +3537,12 @@
       </c>
       <c r="H24" s="100" t="inlineStr">
         <is>
-          <t>5.01***</t>
+          <t>5.01</t>
         </is>
       </c>
       <c r="I24" s="100" t="inlineStr">
         <is>
-          <t>&lt;.001</t>
+          <t>&lt;.001***</t>
         </is>
       </c>
       <c r="J24" s="100" t="inlineStr">
@@ -3557,7 +3557,7 @@
       </c>
       <c r="L24" s="100" t="inlineStr">
         <is>
-          <t>.377</t>
+          <t>.188</t>
         </is>
       </c>
       <c r="M24" s="101" t="inlineStr"/>
@@ -3565,7 +3565,7 @@
     <row r="25" ht="15.75" customHeight="1" thickTop="1">
       <c r="A25" s="30" t="inlineStr">
         <is>
-          <t>Note: Significance levels: *p&lt;.05; **p&lt;.01; ***p&lt;.001; One-tailed test: †. Results: U = Utah, NU = Not Utah (variation results show which group has the larger variance).</t>
+          <t>Note: Significance levels: *p&lt;.05; **p&lt;.01; ***p&lt;.001. All tests are one-tailed. Results: NU = Not Utah, U = Utah (for variation, the group with the larger variance is shown as greater).</t>
         </is>
       </c>
     </row>
@@ -4500,17 +4500,17 @@
       </c>
       <c r="G19" s="97" t="inlineStr">
         <is>
-          <t>-1.97*</t>
+          <t>-1.97</t>
         </is>
       </c>
       <c r="H19" s="97" t="inlineStr">
         <is>
-          <t>.049</t>
+          <t>.025*</t>
         </is>
       </c>
       <c r="I19" s="98" t="inlineStr">
         <is>
-          <t>Female Not Utah &gt; Female Utah</t>
+          <t>FU &lt; FNU</t>
         </is>
       </c>
     </row>
@@ -4544,7 +4544,7 @@
       </c>
       <c r="H20" s="97" t="inlineStr">
         <is>
-          <t>.920</t>
+          <t>.460</t>
         </is>
       </c>
       <c r="I20" s="98" t="inlineStr"/>
@@ -4574,17 +4574,17 @@
       </c>
       <c r="G21" s="97" t="inlineStr">
         <is>
-          <t>-2.16*</t>
+          <t>-2.16</t>
         </is>
       </c>
       <c r="H21" s="97" t="inlineStr">
         <is>
-          <t>.031</t>
+          <t>.015*</t>
         </is>
       </c>
       <c r="I21" s="98" t="inlineStr">
         <is>
-          <t>Female Not Utah &gt; Female Utah</t>
+          <t>FU &lt; FNU</t>
         </is>
       </c>
     </row>
@@ -4613,17 +4613,17 @@
       </c>
       <c r="G22" s="97" t="inlineStr">
         <is>
-          <t>-1.65†</t>
+          <t>-1.65</t>
         </is>
       </c>
       <c r="H22" s="97" t="inlineStr">
         <is>
-          <t>.099</t>
+          <t>.050*</t>
         </is>
       </c>
       <c r="I22" s="98" t="inlineStr">
         <is>
-          <t>Female Not Utah &gt; Female Utah</t>
+          <t>FU &lt; FNU</t>
         </is>
       </c>
     </row>
@@ -4652,17 +4652,17 @@
       </c>
       <c r="G23" s="97" t="inlineStr">
         <is>
-          <t>2.20*</t>
+          <t>2.20</t>
         </is>
       </c>
       <c r="H23" s="97" t="inlineStr">
         <is>
-          <t>.028</t>
+          <t>.014*</t>
         </is>
       </c>
       <c r="I23" s="98" t="inlineStr">
         <is>
-          <t>Female Utah &gt; Female Not Utah</t>
+          <t>FU &gt; FNU</t>
         </is>
       </c>
     </row>
@@ -4895,7 +4895,7 @@
     <row r="38" ht="15.75" customHeight="1" thickTop="1">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Note: Significance levels: *p&lt;.05; **p&lt;.01; ***p&lt;.001; One-tailed test: †</t>
+          <t>Note: Significance levels: *p&lt;.05; **p&lt;.01; ***p&lt;.001. All tests are one-tailed. Results: FU = Female Utah, FNU = Female Not Utah.</t>
         </is>
       </c>
     </row>

</xml_diff>